<commit_message>
feat: add remaining graphs + statistics indicators
</commit_message>
<xml_diff>
--- a/docs/Projeto Análise de Dados Vinhos.xlsx
+++ b/docs/Projeto Análise de Dados Vinhos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20384"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\gabiru\projeto-vinhos\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\gabiru\github\wines-mag-py\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6238DE9-3DB8-4A06-8051-C9B9AC33B6B6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E77C3190-F8F3-49AA-95E9-E3B68B78F0F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="17490" windowHeight="7980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Perguntas" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="53">
   <si>
     <t>N</t>
   </si>
@@ -272,8 +272,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="11">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -639,14 +639,14 @@
       <c r="B15" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E15" s="8" t="s">
-        <v>52</v>
-      </c>
     </row>
     <row r="16" spans="1:5">
       <c r="B16" s="8" t="s">
         <v>17</v>
       </c>
+      <c r="E16" s="5" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="17" spans="2:5">
       <c r="B17" s="3" t="s">
@@ -665,16 +665,16 @@
       <c r="B19" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="E19" s="9" t="s">
-        <v>25</v>
+      <c r="E19" s="10" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="20" spans="2:5">
       <c r="B20" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="E20" s="9" t="s">
-        <v>37</v>
+      <c r="E20" s="10" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="21" spans="2:5">
@@ -686,16 +686,10 @@
       <c r="B22" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E22" s="10" t="s">
-        <v>39</v>
-      </c>
     </row>
     <row r="23" spans="2:5">
       <c r="B23" s="3" t="s">
         <v>24</v>
-      </c>
-      <c r="E23" s="10" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="24" spans="2:5">

</xml_diff>